<commit_message>
Created BroilerHerd class and implemented calculation of herd structure and meat production
</commit_message>
<xml_diff>
--- a/data/prod_parameters/BroilerHerd.xlsx
+++ b/data/prod_parameters/BroilerHerd.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="122">
   <si>
     <t>Höns</t>
   </si>
@@ -280,9 +280,6 @@
     <t>Applies to broilers. LWG = live weight gain</t>
   </si>
   <si>
-    <t>Per inserted (grand)parent hen, includes feed for roasters (1 roaster per 12.5 hens)</t>
-  </si>
-  <si>
     <t>breeder_feed</t>
   </si>
   <si>
@@ -374,6 +371,27 @@
   </si>
   <si>
     <t>% of DM</t>
+  </si>
+  <si>
+    <t>Per inserted (grand)parent hen, includes feed for roosters (1 roaster per 12.5 hens)</t>
+  </si>
+  <si>
+    <t>slaughter_age</t>
+  </si>
+  <si>
+    <t>days</t>
+  </si>
+  <si>
+    <t>Tynelius (2008)</t>
+  </si>
+  <si>
+    <t>parent hens 24 weeks growing + 40 weeks egg laying. Assuming same slaughter age for roosters</t>
+  </si>
+  <si>
+    <t>broiler places</t>
+  </si>
+  <si>
+    <t>f_sub_system</t>
   </si>
 </sst>
 </file>
@@ -938,44 +956,47 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="15.7109375" customWidth="1"/>
-    <col min="4" max="4" width="27" customWidth="1"/>
-    <col min="5" max="5" width="8.42578125" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" customWidth="1"/>
-    <col min="7" max="7" width="44.140625" customWidth="1"/>
-    <col min="8" max="8" width="13.28515625" customWidth="1"/>
+    <col min="1" max="4" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="27" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" customWidth="1"/>
+    <col min="8" max="8" width="44.140625" customWidth="1"/>
+    <col min="9" max="9" width="13.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>67</v>
       </c>
       <c r="B1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" t="s">
         <v>31</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>68</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>69</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>25</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>24</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>70</v>
       </c>
@@ -986,75 +1007,86 @@
       <c r="F2" s="13"/>
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D3" t="s">
+      <c r="I2" s="13"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E3" t="s">
         <v>20</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>8.5</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>26</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D4" t="s">
-        <v>50</v>
-      </c>
-      <c r="E4">
-        <v>24</v>
-      </c>
-      <c r="F4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E5">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4">
+        <v>150</v>
+      </c>
+      <c r="G4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" t="s">
+        <v>45</v>
+      </c>
+      <c r="I4" t="s">
         <v>40</v>
       </c>
-      <c r="F5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D6" t="s">
-        <v>38</v>
-      </c>
-      <c r="E6">
-        <v>150</v>
-      </c>
-      <c r="F6" t="s">
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5">
+        <v>12.5</v>
+      </c>
+      <c r="G5" t="s">
         <v>26</v>
       </c>
+      <c r="I5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" t="s">
+        <v>116</v>
+      </c>
+      <c r="F6">
+        <v>35</v>
+      </c>
       <c r="G6" t="s">
-        <v>45</v>
-      </c>
-      <c r="H6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D7" t="s">
-        <v>39</v>
-      </c>
-      <c r="E7">
-        <v>12.5</v>
-      </c>
-      <c r="F7" t="s">
-        <v>26</v>
+        <v>117</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E7" t="s">
+        <v>116</v>
+      </c>
+      <c r="F7">
+        <f>(24+40)*7</f>
+        <v>448</v>
+      </c>
+      <c r="G7" t="s">
+        <v>117</v>
       </c>
       <c r="H7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+      <c r="I7" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>72</v>
       </c>
@@ -1065,370 +1097,389 @@
       <c r="F9" s="13"/>
       <c r="G9" s="13"/>
       <c r="H9" s="13"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
+      <c r="I9" s="13"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
         <v>32</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>41</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <v>3</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>29</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D11" t="s">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E11" t="s">
         <v>41</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <v>8</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>29</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>71</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D12" t="s">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" t="s">
         <v>28</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <v>2.2999999999999998</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>29</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B15" t="s">
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
         <v>32</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E16" t="s">
         <v>73</v>
       </c>
-      <c r="E15">
+      <c r="F16">
         <v>1.5</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G16" t="s">
         <v>74</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I16" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
         <v>33</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E17" t="s">
         <v>73</v>
       </c>
-      <c r="E16">
+      <c r="F17">
         <v>4.3</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G17" t="s">
         <v>74</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
         <v>34</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E18" t="s">
         <v>73</v>
       </c>
-      <c r="E17">
+      <c r="F18">
         <v>5</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G18" t="s">
         <v>74</v>
       </c>
-      <c r="H17" t="s">
+      <c r="I18" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D18" t="s">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E19" t="s">
         <v>58</v>
       </c>
-      <c r="E18" s="10">
+      <c r="F19" s="10">
         <f>1/0.7</f>
         <v>1.4285714285714286</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G19" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E19" s="10"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="13" t="s">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F20" s="10"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="13"/>
-      <c r="H20" s="13"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D21" t="s">
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="13"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E22" t="s">
         <v>59</v>
       </c>
-      <c r="E21">
+      <c r="F22">
         <v>1.52</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G22" t="s">
         <v>78</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H22" t="s">
         <v>83</v>
       </c>
-      <c r="H21" t="s">
+      <c r="I22" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D22" t="s">
-        <v>85</v>
-      </c>
-      <c r="E22">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E23" t="s">
+        <v>84</v>
+      </c>
+      <c r="F23">
         <v>48</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G23" t="s">
         <v>79</v>
       </c>
-      <c r="G22" t="s">
-        <v>84</v>
-      </c>
-      <c r="H22" t="s">
+      <c r="H23" t="s">
+        <v>115</v>
+      </c>
+      <c r="I23" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="17" t="s">
-        <v>115</v>
-      </c>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D25" s="14" t="s">
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
+      <c r="G25" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="H25" s="13"/>
+      <c r="I25" s="13"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E26" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="E25" s="14">
+      <c r="F26" s="14">
         <v>0</v>
       </c>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14" t="s">
+      <c r="G26" s="14"/>
+      <c r="H26" s="14" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>32</v>
-      </c>
-      <c r="B26" t="s">
-        <v>86</v>
-      </c>
-      <c r="D26" t="s">
-        <v>81</v>
-      </c>
-      <c r="E26" s="11">
-        <v>56.465302046929608</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>32</v>
       </c>
-      <c r="B27" t="s">
-        <v>87</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="C27" t="s">
+        <v>85</v>
+      </c>
+      <c r="E27" t="s">
         <v>81</v>
       </c>
-      <c r="E27" s="11">
-        <v>4.6396314618980625</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F27" s="11">
+        <v>56.465302046929608</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>32</v>
       </c>
-      <c r="B28" t="s">
-        <v>88</v>
-      </c>
-      <c r="D28" t="s">
+      <c r="C28" t="s">
+        <v>86</v>
+      </c>
+      <c r="E28" t="s">
         <v>81</v>
       </c>
-      <c r="E28" s="11">
-        <v>2.8627513275541236</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F28" s="11">
+        <v>4.6396314618980625</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>32</v>
       </c>
-      <c r="B29" t="s">
-        <v>89</v>
-      </c>
-      <c r="D29" t="s">
+      <c r="C29" t="s">
+        <v>87</v>
+      </c>
+      <c r="E29" t="s">
         <v>81</v>
       </c>
-      <c r="E29" s="11">
-        <v>6.2258884400671732</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F29" s="11">
+        <v>2.8627513275541236</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>32</v>
       </c>
-      <c r="B30" t="s">
-        <v>90</v>
-      </c>
-      <c r="D30" t="s">
+      <c r="C30" t="s">
+        <v>88</v>
+      </c>
+      <c r="E30" t="s">
         <v>81</v>
       </c>
-      <c r="E30" s="11">
-        <v>17.768801343439385</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F30" s="11">
+        <v>6.2258884400671732</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>32</v>
       </c>
-      <c r="B31" t="s">
-        <v>91</v>
-      </c>
-      <c r="D31" t="s">
+      <c r="C31" t="s">
+        <v>89</v>
+      </c>
+      <c r="E31" t="s">
         <v>81</v>
       </c>
-      <c r="E31" s="11">
-        <v>2.8593473426224301</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F31" s="11">
+        <v>17.768801343439385</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>32</v>
       </c>
-      <c r="B32" t="s">
-        <v>92</v>
-      </c>
-      <c r="D32" t="s">
+      <c r="C32" t="s">
+        <v>90</v>
+      </c>
+      <c r="E32" t="s">
         <v>81</v>
       </c>
-      <c r="E32" s="11">
-        <v>0.61271728770480649</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F32" s="11">
+        <v>2.8593473426224301</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>32</v>
       </c>
-      <c r="B33" t="s">
-        <v>101</v>
-      </c>
-      <c r="D33" t="s">
+      <c r="C33" t="s">
+        <v>91</v>
+      </c>
+      <c r="E33" t="s">
         <v>81</v>
       </c>
-      <c r="E33" s="11">
-        <v>2.6653202015159083</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F33" s="11">
+        <v>0.61271728770480649</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>32</v>
       </c>
-      <c r="B34" t="s">
-        <v>93</v>
-      </c>
-      <c r="D34" t="s">
+      <c r="C34" t="s">
+        <v>100</v>
+      </c>
+      <c r="E34" t="s">
         <v>81</v>
       </c>
-      <c r="E34" s="11">
-        <v>1.5885263014569055</v>
-      </c>
-      <c r="G34" s="15" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F34" s="11">
+        <v>2.6653202015159083</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>32</v>
       </c>
-      <c r="B35" t="s">
-        <v>95</v>
-      </c>
-      <c r="D35" t="s">
+      <c r="C35" t="s">
+        <v>92</v>
+      </c>
+      <c r="E35" t="s">
         <v>81</v>
       </c>
-      <c r="E35" s="11">
-        <v>2.0423909590160214</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F35" s="11">
+        <v>1.5885263014569055</v>
+      </c>
+      <c r="H35" s="15" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>32</v>
       </c>
-      <c r="B36" t="s">
-        <v>96</v>
-      </c>
-      <c r="D36" t="s">
+      <c r="C36" t="s">
+        <v>94</v>
+      </c>
+      <c r="E36" t="s">
         <v>81</v>
       </c>
-      <c r="E36" s="11">
+      <c r="F36" s="11">
+        <v>2.0423909590160214</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>32</v>
+      </c>
+      <c r="C37" t="s">
+        <v>95</v>
+      </c>
+      <c r="E37" t="s">
+        <v>81</v>
+      </c>
+      <c r="F37" s="11">
         <v>2.2693232877955793</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:V47"/>
+  <dimension ref="B2:V48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.28515625" customWidth="1"/>
@@ -1649,6 +1700,18 @@
       </c>
     </row>
     <row r="8" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" t="s">
+        <v>116</v>
+      </c>
+      <c r="D8">
+        <v>35</v>
+      </c>
+      <c r="E8" t="s">
+        <v>117</v>
+      </c>
       <c r="O8" s="5" t="s">
         <v>3</v>
       </c>
@@ -1674,21 +1737,6 @@
       </c>
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9">
-        <v>3</v>
-      </c>
-      <c r="E9" t="s">
-        <v>29</v>
-      </c>
-      <c r="G9" t="s">
-        <v>22</v>
-      </c>
       <c r="O9" s="5" t="s">
         <v>4</v>
       </c>
@@ -1714,17 +1762,20 @@
       </c>
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>32</v>
+      </c>
       <c r="C10" t="s">
         <v>41</v>
       </c>
       <c r="D10">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E10" t="s">
         <v>29</v>
       </c>
       <c r="G10" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="O10" s="5"/>
       <c r="P10" s="5"/>
@@ -1737,16 +1788,16 @@
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="D11">
-        <v>2.2999999999999998</v>
+        <v>8</v>
       </c>
       <c r="E11" t="s">
         <v>29</v>
       </c>
       <c r="G11" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="O11" s="7" t="s">
         <v>13</v>
@@ -1760,6 +1811,18 @@
       <c r="V11" s="9"/>
     </row>
     <row r="12" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E12" t="s">
+        <v>29</v>
+      </c>
+      <c r="G12" t="s">
+        <v>30</v>
+      </c>
       <c r="O12" s="5" t="s">
         <v>5</v>
       </c>
@@ -1810,21 +1873,6 @@
       </c>
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" t="s">
-        <v>73</v>
-      </c>
-      <c r="D14">
-        <v>1.5</v>
-      </c>
-      <c r="E14" t="s">
-        <v>74</v>
-      </c>
-      <c r="G14" t="s">
-        <v>30</v>
-      </c>
       <c r="O14" s="5" t="s">
         <v>7</v>
       </c>
@@ -1851,19 +1899,19 @@
     </row>
     <row r="15" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C15" t="s">
         <v>73</v>
       </c>
       <c r="D15">
-        <v>4.3</v>
+        <v>1.5</v>
       </c>
       <c r="E15" t="s">
         <v>74</v>
       </c>
       <c r="G15" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="O15" s="5" t="s">
         <v>8</v>
@@ -1891,19 +1939,19 @@
     </row>
     <row r="16" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C16" t="s">
         <v>73</v>
       </c>
       <c r="D16">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="E16" t="s">
         <v>74</v>
       </c>
       <c r="G16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O16" s="5" t="s">
         <v>9</v>
@@ -1930,15 +1978,20 @@
       </c>
     </row>
     <row r="17" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>34</v>
+      </c>
       <c r="C17" t="s">
-        <v>58</v>
-      </c>
-      <c r="D17" s="10">
-        <f>1/0.7</f>
-        <v>1.4285714285714286</v>
+        <v>73</v>
+      </c>
+      <c r="D17">
+        <v>5</v>
       </c>
       <c r="E17" t="s">
-        <v>57</v>
+        <v>74</v>
+      </c>
+      <c r="G17" t="s">
+        <v>37</v>
       </c>
       <c r="O17" s="5" t="s">
         <v>10</v>
@@ -1965,6 +2018,16 @@
       </c>
     </row>
     <row r="18" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
+        <v>58</v>
+      </c>
+      <c r="D18" s="10">
+        <f>1/0.7</f>
+        <v>1.4285714285714286</v>
+      </c>
+      <c r="E18" t="s">
+        <v>57</v>
+      </c>
       <c r="O18" s="5" t="s">
         <v>11</v>
       </c>
@@ -1990,18 +2053,6 @@
       </c>
     </row>
     <row r="19" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="C19" t="s">
-        <v>59</v>
-      </c>
-      <c r="D19">
-        <v>1.52</v>
-      </c>
-      <c r="E19" t="s">
-        <v>61</v>
-      </c>
-      <c r="G19" t="s">
-        <v>63</v>
-      </c>
       <c r="O19" s="5" t="s">
         <v>12</v>
       </c>
@@ -2028,19 +2079,16 @@
     </row>
     <row r="20" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D20">
-        <v>48</v>
+        <v>1.52</v>
       </c>
       <c r="E20" t="s">
-        <v>62</v>
-      </c>
-      <c r="F20" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="G20" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="O20" s="7" t="s">
         <v>14</v>
@@ -2054,6 +2102,21 @@
       <c r="V20" s="9"/>
     </row>
     <row r="21" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
+        <v>60</v>
+      </c>
+      <c r="D21">
+        <v>48</v>
+      </c>
+      <c r="E21" t="s">
+        <v>62</v>
+      </c>
+      <c r="F21" t="s">
+        <v>65</v>
+      </c>
+      <c r="G21" t="s">
+        <v>64</v>
+      </c>
       <c r="O21" s="5" t="s">
         <v>5</v>
       </c>
@@ -2079,9 +2142,6 @@
       </c>
     </row>
     <row r="22" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
-        <v>42</v>
-      </c>
       <c r="O22" s="5" t="s">
         <v>6</v>
       </c>
@@ -2108,11 +2168,7 @@
     </row>
     <row r="23" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" s="1">
-        <f>V8</f>
-        <v>12677624</v>
+        <v>42</v>
       </c>
       <c r="O23" s="5" t="s">
         <v>7</v>
@@ -2139,8 +2195,15 @@
       </c>
     </row>
     <row r="24" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B24" s="2" t="s">
-        <v>53</v>
+      <c r="B24" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" s="1">
+        <f>V8</f>
+        <v>12677624</v>
+      </c>
+      <c r="D24" t="s">
+        <v>120</v>
       </c>
       <c r="O24" s="5" t="s">
         <v>8</v>
@@ -2167,12 +2230,8 @@
       </c>
     </row>
     <row r="25" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B25" t="s">
-        <v>32</v>
-      </c>
-      <c r="C25" s="1">
-        <f>C23</f>
-        <v>12677624</v>
+      <c r="B25" s="2" t="s">
+        <v>53</v>
       </c>
       <c r="O25" s="5" t="s">
         <v>9</v>
@@ -2200,11 +2259,11 @@
     </row>
     <row r="26" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="C26" s="1">
-        <f>C32*(D$4+D$5)/52.2</f>
-        <v>957386.23132878006</v>
+        <f>C24</f>
+        <v>12677624</v>
       </c>
       <c r="O26" s="5" t="s">
         <v>10</v>
@@ -2232,11 +2291,11 @@
     </row>
     <row r="27" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C27" s="1">
         <f>C33*(D$4+D$5)/52.2</f>
-        <v>76590.898506302401</v>
+        <v>957386.23132878006</v>
       </c>
       <c r="O27" s="5" t="s">
         <v>11</v>
@@ -2264,11 +2323,11 @@
     </row>
     <row r="28" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C28" s="1">
         <f>C34*(D$4+D$5)/52.2</f>
-        <v>6937.5813864404345</v>
+        <v>76590.898506302401</v>
       </c>
       <c r="O28" s="5" t="s">
         <v>12</v>
@@ -2296,18 +2355,21 @@
     </row>
     <row r="29" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C29" s="1">
         <f>C35*(D$4+D$5)/52.2</f>
+        <v>6937.5813864404345</v>
+      </c>
+    </row>
+    <row r="30" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>49</v>
+      </c>
+      <c r="C30" s="1">
+        <f>C36*(D$4+D$5)/52.2</f>
         <v>2312.5271288134782</v>
       </c>
-    </row>
-    <row r="30" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B30" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C30" s="1"/>
       <c r="O30" t="s">
         <v>27</v>
       </c>
@@ -2337,13 +2399,10 @@
       </c>
     </row>
     <row r="31" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B31" t="s">
-        <v>32</v>
-      </c>
-      <c r="C31" s="1">
-        <f>C25*D3</f>
-        <v>107759804</v>
-      </c>
+      <c r="B31" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C31" s="1"/>
       <c r="O31" t="s">
         <v>35</v>
       </c>
@@ -2375,11 +2434,11 @@
     </row>
     <row r="32" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="C32" s="1">
-        <f>C31/D6/(1-D10/100)</f>
-        <v>780868.14492753625</v>
+        <f>C24*D3</f>
+        <v>107759804</v>
       </c>
       <c r="P32" s="10">
         <f t="shared" si="1"/>
@@ -2409,183 +2468,192 @@
     </row>
     <row r="33" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C33" s="1">
-        <f>C32/D7</f>
-        <v>62469.451594202903</v>
+        <f>C32/D6/(1-D11/100)</f>
+        <v>780868.14492753625</v>
+      </c>
+      <c r="E33" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="34" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C34" s="1">
-        <f>C32/D6/(1-D10/100)</f>
-        <v>5658.4648183154795</v>
+        <f>C33/D7</f>
+        <v>62469.451594202903</v>
       </c>
       <c r="P34" s="1">
-        <f>$C$37/$C$23*P8/1000</f>
+        <f>$C$38/$C$24*P8/1000</f>
         <v>93244.426457059992</v>
       </c>
       <c r="Q34" s="1">
-        <f t="shared" ref="Q34:V34" si="2">$C$37/$C$23*Q8/1000</f>
+        <f>$C$38/$C$24*Q8/1000</f>
         <v>98229.811301909998</v>
       </c>
       <c r="R34" s="1">
-        <f t="shared" si="2"/>
+        <f>$C$38/$C$24*R8/1000</f>
         <v>104179.173620945</v>
       </c>
       <c r="S34" s="1">
-        <f t="shared" si="2"/>
+        <f>$C$38/$C$24*S8/1000</f>
         <v>106530.905211235</v>
       </c>
       <c r="T34" s="1">
-        <f t="shared" si="2"/>
+        <f>$C$38/$C$24*T8/1000</f>
         <v>108430.12667264999</v>
       </c>
       <c r="U34" s="1"/>
       <c r="V34" s="1">
-        <f t="shared" si="2"/>
+        <f>$C$38/$C$24*V8/1000</f>
         <v>102122.88865276</v>
       </c>
     </row>
     <row r="35" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C35" s="1">
-        <f>C34/D9</f>
-        <v>1886.1549394384931</v>
+        <f>C33/D6/(1-D11/100)</f>
+        <v>5658.4648183154795</v>
       </c>
       <c r="P35" s="12">
         <f>P34/P13</f>
         <v>0.93908358552022797</v>
       </c>
       <c r="Q35" s="12">
-        <f t="shared" ref="Q35:V35" si="3">Q34/Q13</f>
+        <f t="shared" ref="Q35:V35" si="2">Q34/Q13</f>
         <v>0.98205613438758688</v>
       </c>
       <c r="R35" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1.0576293121065203</v>
       </c>
       <c r="S35" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1.0297754156643528</v>
       </c>
       <c r="T35" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1.0116088739410678</v>
       </c>
       <c r="U35" s="12"/>
       <c r="V35" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1.0042438689534616</v>
       </c>
     </row>
     <row r="36" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B36" s="2" t="s">
+      <c r="B36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C36" s="1">
+        <f>C35/D10</f>
+        <v>1886.1549394384931</v>
+      </c>
+    </row>
+    <row r="37" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B37" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C36" s="1"/>
-    </row>
-    <row r="37" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B37" t="s">
-        <v>32</v>
-      </c>
-      <c r="C37" s="1">
-        <f>C31-C43</f>
-        <v>102122888.65276</v>
-      </c>
+      <c r="C37" s="1"/>
     </row>
     <row r="38" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="C38" s="1">
         <f>C32-C44</f>
-        <v>701875.52338666667</v>
-      </c>
-      <c r="E38" t="s">
-        <v>66</v>
+        <v>102122888.65276</v>
       </c>
     </row>
     <row r="39" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C39" s="1">
         <f>C33-C45</f>
-        <v>56150.041870933339</v>
+        <v>701875.52338666667</v>
       </c>
     </row>
     <row r="40" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C40" s="1">
         <f>C34-C46</f>
-        <v>5086.0545172946859</v>
+        <v>56150.041870933339</v>
       </c>
     </row>
     <row r="41" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C41" s="1">
         <f>C35-C47</f>
+        <v>5086.0545172946859</v>
+      </c>
+    </row>
+    <row r="42" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B42" t="s">
+        <v>49</v>
+      </c>
+      <c r="C42" s="1">
+        <f>C36-C48</f>
         <v>1695.3515057648951</v>
       </c>
     </row>
-    <row r="42" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B42" s="2" t="s">
+    <row r="43" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B43" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C42" s="1"/>
-    </row>
-    <row r="43" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B43" t="s">
-        <v>32</v>
-      </c>
-      <c r="C43" s="1">
-        <f>C31*(D$9/100) + C31*(1-D$9/100)*(D$11/100)</f>
-        <v>5636915.34724</v>
-      </c>
+      <c r="C43" s="1"/>
     </row>
     <row r="44" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="C44" s="1">
-        <f>C32*(D$10/100) + C32*(1-D$10/100)*(D$11/100)</f>
-        <v>78992.621540869572</v>
+        <f>C32*(D$10/100) + C32*(1-D$10/100)*(D$12/100)</f>
+        <v>5636915.34724</v>
       </c>
     </row>
     <row r="45" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C45" s="1">
-        <f t="shared" ref="C45:C47" si="4">C33*(D$10/100) + C33*(1-D$10/100)*(D$11/100)</f>
-        <v>6319.4097232695658</v>
+        <f>C33*(D$11/100) + C33*(1-D$11/100)*(D$12/100)</f>
+        <v>78992.621540869572</v>
       </c>
     </row>
     <row r="46" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C46" s="1">
-        <f t="shared" si="4"/>
-        <v>572.4103010207939</v>
+        <f>C34*(D$11/100) + C34*(1-D$11/100)*(D$12/100)</f>
+        <v>6319.4097232695658</v>
       </c>
     </row>
     <row r="47" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
+        <v>48</v>
+      </c>
+      <c r="C47" s="1">
+        <f>C35*(D$11/100) + C35*(1-D$11/100)*(D$12/100)</f>
+        <v>572.4103010207939</v>
+      </c>
+    </row>
+    <row r="48" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
         <v>49</v>
       </c>
-      <c r="C47" s="1">
-        <f t="shared" si="4"/>
+      <c r="C48" s="1">
+        <f>C36*(D$11/100) + C36*(1-D$11/100)*(D$12/100)</f>
         <v>190.80343367359797</v>
       </c>
     </row>
@@ -2607,41 +2675,41 @@
   <sheetData>
     <row r="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="F1" t="s">
+        <v>111</v>
+      </c>
+      <c r="I1" t="s">
         <v>112</v>
-      </c>
-      <c r="I1" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F2" t="s">
         <v>109</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>110</v>
       </c>
-      <c r="G2" t="s">
-        <v>111</v>
-      </c>
       <c r="H2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I2" t="s">
+        <v>109</v>
+      </c>
+      <c r="J2" t="s">
         <v>110</v>
       </c>
-      <c r="J2" t="s">
-        <v>111</v>
-      </c>
       <c r="K2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D3">
         <v>0.87</v>
@@ -2656,10 +2724,10 @@
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D4">
         <v>0.87</v>
@@ -2674,10 +2742,10 @@
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D5">
         <v>0.87</v>
@@ -2692,10 +2760,10 @@
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D6">
         <v>0.93</v>
@@ -2710,10 +2778,10 @@
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D7">
         <v>0.87</v>
@@ -2728,10 +2796,10 @@
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D8">
         <v>0.9</v>
@@ -2746,10 +2814,10 @@
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D9">
         <v>0.9</v>
@@ -2764,10 +2832,10 @@
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D10">
         <v>0.87</v>
@@ -2782,10 +2850,10 @@
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C11" t="s">
         <v>93</v>
-      </c>
-      <c r="C11" t="s">
-        <v>94</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -2800,10 +2868,10 @@
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -2818,10 +2886,10 @@
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C13" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -2836,7 +2904,7 @@
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
       <c r="E15" s="16" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F15" s="10">
         <f t="shared" ref="F15:G15" si="1">SUMPRODUCT(F$3:F$13/100,$D$3:$D$13)</f>

</xml_diff>

<commit_message>
Feed demand + manure mgmt implemented for broilers
</commit_message>
<xml_diff>
--- a/data/prod_parameters/BroilerHerd.xlsx
+++ b/data/prod_parameters/BroilerHerd.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="default" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="123">
   <si>
     <t>Höns</t>
   </si>
@@ -277,12 +277,6 @@
     <t>Fallback</t>
   </si>
   <si>
-    <t>Applies to broilers. LWG = live weight gain</t>
-  </si>
-  <si>
-    <t>breeder_feed</t>
-  </si>
-  <si>
     <t>wheat</t>
   </si>
   <si>
@@ -392,6 +386,15 @@
   </si>
   <si>
     <t>f_sub_system</t>
+  </si>
+  <si>
+    <t>feed_per_animal</t>
+  </si>
+  <si>
+    <t>LWG = live weight gain</t>
+  </si>
+  <si>
+    <t>Ration DM (excl. minerals and amino acids):</t>
   </si>
 </sst>
 </file>
@@ -956,7 +959,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="15.7109375" customWidth="1"/>
@@ -972,7 +975,7 @@
         <v>67</v>
       </c>
       <c r="B1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C1" t="s">
         <v>31</v>
@@ -1059,31 +1062,31 @@
         <v>32</v>
       </c>
       <c r="E6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F6">
         <v>35</v>
       </c>
       <c r="G6" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F7">
         <f>(24+40)*7</f>
         <v>448</v>
       </c>
       <c r="G7" t="s">
+        <v>115</v>
+      </c>
+      <c r="H7" t="s">
         <v>117</v>
       </c>
-      <c r="H7" t="s">
-        <v>119</v>
-      </c>
       <c r="I7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -1254,6 +1257,9 @@
       <c r="I21" s="13"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
+        <v>32</v>
+      </c>
       <c r="E22" t="s">
         <v>59</v>
       </c>
@@ -1264,15 +1270,18 @@
         <v>78</v>
       </c>
       <c r="H22" t="s">
-        <v>83</v>
+        <v>121</v>
       </c>
       <c r="I22" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C23" t="s">
+        <v>33</v>
+      </c>
       <c r="E23" t="s">
-        <v>84</v>
+        <v>120</v>
       </c>
       <c r="F23">
         <v>48</v>
@@ -1281,195 +1290,166 @@
         <v>79</v>
       </c>
       <c r="H23" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I23" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="13" t="s">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C24" t="s">
+        <v>34</v>
+      </c>
+      <c r="E24" t="s">
+        <v>120</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="17" t="s">
-        <v>114</v>
-      </c>
-      <c r="H25" s="13"/>
-      <c r="I25" s="13"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="E26" s="14" t="s">
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="H26" s="13"/>
+      <c r="I26" s="13"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E27" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="F26" s="14">
+      <c r="F27" s="14">
         <v>0</v>
       </c>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14" t="s">
+      <c r="G27" s="14"/>
+      <c r="H27" s="14" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>32</v>
-      </c>
-      <c r="C27" t="s">
-        <v>85</v>
-      </c>
-      <c r="E27" t="s">
-        <v>81</v>
-      </c>
-      <c r="F27" s="11">
-        <v>56.465302046929608</v>
-      </c>
-    </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>32</v>
-      </c>
-      <c r="C28" t="s">
-        <v>86</v>
+      <c r="D28" t="s">
+        <v>83</v>
       </c>
       <c r="E28" t="s">
         <v>81</v>
       </c>
       <c r="F28" s="11">
-        <v>4.6396314618980625</v>
+        <v>59.009628610729031</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>32</v>
-      </c>
-      <c r="C29" t="s">
-        <v>87</v>
+      <c r="D29" t="s">
+        <v>84</v>
       </c>
       <c r="E29" t="s">
         <v>81</v>
       </c>
       <c r="F29" s="11">
-        <v>2.8627513275541236</v>
+        <v>4.8486932599724906</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>32</v>
-      </c>
-      <c r="C30" t="s">
-        <v>88</v>
+      <c r="D30" t="s">
+        <v>85</v>
       </c>
       <c r="E30" t="s">
         <v>81</v>
       </c>
       <c r="F30" s="11">
-        <v>6.2258884400671732</v>
+        <v>2.9917469050894088</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>32</v>
-      </c>
-      <c r="C31" t="s">
-        <v>89</v>
+      <c r="D31" t="s">
+        <v>86</v>
       </c>
       <c r="E31" t="s">
         <v>81</v>
       </c>
       <c r="F31" s="11">
-        <v>17.768801343439385</v>
+        <v>6.5064269790826748</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>32</v>
-      </c>
-      <c r="C32" t="s">
-        <v>90</v>
+      <c r="D32" t="s">
+        <v>87</v>
       </c>
       <c r="E32" t="s">
         <v>81</v>
       </c>
       <c r="F32" s="11">
-        <v>2.8593473426224301</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>32</v>
-      </c>
-      <c r="C33" t="s">
-        <v>91</v>
+        <v>18.569463548830814</v>
+      </c>
+    </row>
+    <row r="33" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D33" t="s">
+        <v>88</v>
       </c>
       <c r="E33" t="s">
         <v>81</v>
       </c>
       <c r="F33" s="11">
-        <v>0.61271728770480649</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>32</v>
-      </c>
-      <c r="C34" t="s">
-        <v>100</v>
+        <v>2.9881895365934641</v>
+      </c>
+    </row>
+    <row r="34" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D34" t="s">
+        <v>89</v>
       </c>
       <c r="E34" t="s">
         <v>81</v>
       </c>
       <c r="F34" s="11">
-        <v>2.6653202015159083</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>32</v>
-      </c>
-      <c r="C35" t="s">
-        <v>92</v>
+        <v>0.64032632927002808</v>
+      </c>
+    </row>
+    <row r="35" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D35" t="s">
+        <v>98</v>
       </c>
       <c r="E35" t="s">
         <v>81</v>
       </c>
       <c r="F35" s="11">
-        <v>1.5885263014569055</v>
-      </c>
-      <c r="H35" s="15" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>32</v>
-      </c>
-      <c r="C36" t="s">
-        <v>94</v>
+        <v>2.7854195323246222</v>
+      </c>
+    </row>
+    <row r="36" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D36" t="s">
+        <v>90</v>
       </c>
       <c r="E36" t="s">
         <v>81</v>
       </c>
       <c r="F36" s="11">
-        <v>2.0423909590160214</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>32</v>
-      </c>
-      <c r="C37" t="s">
-        <v>95</v>
-      </c>
-      <c r="E37" t="s">
-        <v>81</v>
-      </c>
-      <c r="F37" s="11">
-        <v>2.2693232877955793</v>
-      </c>
+        <v>1.66010529810748</v>
+      </c>
+      <c r="H36" s="15" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="37" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D37" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="F37" s="11"/>
+    </row>
+    <row r="38" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D38" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="F38" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1704,13 +1684,13 @@
         <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D8">
         <v>35</v>
       </c>
       <c r="E8" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="O8" s="5" t="s">
         <v>3</v>
@@ -2170,6 +2150,7 @@
       <c r="B23" t="s">
         <v>42</v>
       </c>
+      <c r="F23" s="1"/>
       <c r="O23" s="5" t="s">
         <v>7</v>
       </c>
@@ -2203,8 +2184,9 @@
         <v>12677624</v>
       </c>
       <c r="D24" t="s">
-        <v>120</v>
-      </c>
+        <v>118</v>
+      </c>
+      <c r="F24" s="1"/>
       <c r="O24" s="5" t="s">
         <v>8</v>
       </c>
@@ -2403,6 +2385,10 @@
         <v>55</v>
       </c>
       <c r="C31" s="1"/>
+      <c r="F31">
+        <f>C27/((D$4+D$5)/52.2)</f>
+        <v>780868.14492753625</v>
+      </c>
       <c r="O31" t="s">
         <v>35</v>
       </c>
@@ -2666,7 +2652,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:K15"/>
+  <dimension ref="B1:K16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23.5703125" bestFit="1" customWidth="1"/>
@@ -2675,41 +2661,41 @@
   <sheetData>
     <row r="1" spans="2:11" x14ac:dyDescent="0.25">
       <c r="F1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="I1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F2" t="s">
+        <v>107</v>
+      </c>
+      <c r="G2" t="s">
         <v>108</v>
       </c>
-      <c r="F2" t="s">
-        <v>109</v>
-      </c>
-      <c r="G2" t="s">
-        <v>110</v>
-      </c>
       <c r="H2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="I2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="K2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D3">
         <v>0.87</v>
@@ -2718,16 +2704,16 @@
         <v>57.2</v>
       </c>
       <c r="K3" s="11">
-        <f>H3*$D3/H$15</f>
-        <v>56.465302046929608</v>
+        <f>H3*$D3/H$16</f>
+        <v>59.009628610729031</v>
       </c>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D4">
         <v>0.87</v>
@@ -2736,16 +2722,16 @@
         <v>4.7</v>
       </c>
       <c r="K4" s="11">
-        <f>H4*$D4/H$15</f>
-        <v>4.6396314618980625</v>
+        <f t="shared" ref="K4:K11" si="0">H4*$D4/H$16</f>
+        <v>4.8486932599724906</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D5">
         <v>0.87</v>
@@ -2754,16 +2740,16 @@
         <v>2.9</v>
       </c>
       <c r="K5" s="11">
-        <f t="shared" ref="K5:K13" si="0">H5*$D5/H$15</f>
-        <v>2.8627513275541236</v>
+        <f t="shared" si="0"/>
+        <v>2.9917469050894088</v>
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D6">
         <v>0.93</v>
@@ -2773,15 +2759,15 @@
       </c>
       <c r="K6" s="11">
         <f t="shared" si="0"/>
-        <v>6.2258884400671732</v>
+        <v>6.5064269790826748</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D7">
         <v>0.87</v>
@@ -2791,15 +2777,15 @@
       </c>
       <c r="K7" s="11">
         <f t="shared" si="0"/>
-        <v>17.768801343439385</v>
+        <v>18.569463548830814</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C8" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D8">
         <v>0.9</v>
@@ -2809,15 +2795,15 @@
       </c>
       <c r="K8" s="11">
         <f t="shared" si="0"/>
-        <v>2.8593473426224301</v>
+        <v>2.9881895365934641</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C9" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D9">
         <v>0.9</v>
@@ -2827,15 +2813,15 @@
       </c>
       <c r="K9" s="11">
         <f t="shared" si="0"/>
-        <v>0.61271728770480649</v>
+        <v>0.64032632927002808</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C10" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D10">
         <v>0.87</v>
@@ -2845,15 +2831,15 @@
       </c>
       <c r="K10" s="11">
         <f t="shared" si="0"/>
-        <v>2.6653202015159083</v>
+        <v>2.7854195323246222</v>
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C11" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -2863,15 +2849,15 @@
       </c>
       <c r="K11" s="11">
         <f t="shared" si="0"/>
-        <v>1.5885263014569055</v>
+        <v>1.66010529810748</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C12" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -2879,17 +2865,14 @@
       <c r="H12">
         <v>1.8</v>
       </c>
-      <c r="K12" s="11">
-        <f t="shared" si="0"/>
-        <v>2.0423909590160214</v>
-      </c>
+      <c r="K12" s="11"/>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C13" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -2897,14 +2880,11 @@
       <c r="H13">
         <v>2</v>
       </c>
-      <c r="K13" s="11">
-        <f t="shared" si="0"/>
-        <v>2.2693232877955793</v>
-      </c>
+      <c r="K13" s="11"/>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
       <c r="E15" s="16" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F15" s="10">
         <f t="shared" ref="F15:G15" si="1">SUMPRODUCT(F$3:F$13/100,$D$3:$D$13)</f>
@@ -2917,6 +2897,15 @@
       <c r="H15" s="10">
         <f>SUMPRODUCT(H$3:H$13/100,$D$3:$D$13)</f>
         <v>0.88131999999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="E16" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="H16" s="10">
+        <f>SUMPRODUCT(H$3:H$11/100,$D$3:$D$11)</f>
+        <v>0.84331999999999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Manure VS excretion calculation from energy-balance (IPCC Tier 2)
</commit_message>
<xml_diff>
--- a/data/prod_parameters/BroilerHerd.xlsx
+++ b/data/prod_parameters/BroilerHerd.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="126">
   <si>
     <t>Höns</t>
   </si>
@@ -392,6 +392,18 @@
   </si>
   <si>
     <t>Ration DM (excl. minerals and amino acids):</t>
+  </si>
+  <si>
+    <t>start_weight</t>
+  </si>
+  <si>
+    <t>kg LW</t>
+  </si>
+  <si>
+    <t>Statistics Netherlands (2012)</t>
+  </si>
+  <si>
+    <t>???</t>
   </si>
 </sst>
 </file>
@@ -956,7 +968,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="15.7109375" customWidth="1"/>
@@ -1173,272 +1185,329 @@
         <v>32</v>
       </c>
       <c r="D16" t="s">
-        <v>73</v>
+        <v>122</v>
       </c>
       <c r="E16">
-        <v>1.5</v>
+        <f>42/1000</f>
+        <v>4.2000000000000003E-2</v>
       </c>
       <c r="F16" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="H16" t="s">
-        <v>30</v>
+        <v>124</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D17" t="s">
         <v>73</v>
       </c>
       <c r="E17">
-        <v>4.3</v>
+        <v>1.5</v>
       </c>
       <c r="F17" t="s">
         <v>74</v>
       </c>
       <c r="H17" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" t="s">
+        <v>122</v>
+      </c>
+      <c r="E18">
+        <f>42/1000</f>
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="F18" t="s">
+        <v>123</v>
+      </c>
+      <c r="H18" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>33</v>
+      </c>
+      <c r="D19" t="s">
+        <v>73</v>
+      </c>
+      <c r="E19">
+        <v>4.3</v>
+      </c>
+      <c r="F19" t="s">
+        <v>74</v>
+      </c>
+      <c r="H19" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
         <v>34</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D20" t="s">
+        <v>122</v>
+      </c>
+      <c r="E20">
+        <f>42/1000</f>
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="F20" t="s">
+        <v>123</v>
+      </c>
+      <c r="H20" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" t="s">
         <v>73</v>
       </c>
-      <c r="E18">
+      <c r="E21">
         <v>5</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F21" t="s">
         <v>74</v>
       </c>
-      <c r="H18" t="s">
+      <c r="H21" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D19" t="s">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D22" t="s">
         <v>58</v>
       </c>
-      <c r="E19" s="10">
+      <c r="E22" s="10">
         <f>1/0.7</f>
         <v>1.4285714285714286</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F22" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E20" s="10"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
+      <c r="H22" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E23" s="10"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13"/>
-      <c r="H21" s="13"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="13"/>
+      <c r="H24" s="13"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
         <v>32</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D25" t="s">
         <v>59</v>
       </c>
-      <c r="E22">
+      <c r="E25">
         <v>1.52</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F25" t="s">
         <v>78</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G25" t="s">
         <v>120</v>
       </c>
-      <c r="H22" t="s">
+      <c r="H25" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B23" t="s">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
         <v>33</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D26" t="s">
         <v>119</v>
       </c>
-      <c r="E23">
+      <c r="E26">
         <v>48</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F26" t="s">
         <v>79</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G26" t="s">
         <v>113</v>
       </c>
-      <c r="H23" t="s">
+      <c r="H26" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B24" t="s">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
         <v>34</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D27" t="s">
         <v>119</v>
       </c>
-      <c r="E24">
+      <c r="E27">
         <v>0</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F27" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="17" t="s">
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="G26" s="13"/>
-      <c r="H26" s="13"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D27" s="14" t="s">
+      <c r="G29" s="13"/>
+      <c r="H29" s="13"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D30" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="E27" s="14">
+      <c r="E30" s="14">
         <v>0</v>
       </c>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14" t="s">
+      <c r="F30" s="14"/>
+      <c r="G30" s="14" t="s">
         <v>82</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C28" t="s">
-        <v>83</v>
-      </c>
-      <c r="D28" t="s">
-        <v>81</v>
-      </c>
-      <c r="E28" s="11">
-        <v>59.009628610729031</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C29" t="s">
-        <v>84</v>
-      </c>
-      <c r="D29" t="s">
-        <v>81</v>
-      </c>
-      <c r="E29" s="11">
-        <v>4.8486932599724906</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C30" t="s">
-        <v>85</v>
-      </c>
-      <c r="D30" t="s">
-        <v>81</v>
-      </c>
-      <c r="E30" s="11">
-        <v>2.9917469050894088</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C31" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D31" t="s">
         <v>81</v>
       </c>
       <c r="E31" s="11">
-        <v>6.5064269790826748</v>
+        <v>59.009628610729031</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C32" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D32" t="s">
         <v>81</v>
       </c>
       <c r="E32" s="11">
-        <v>18.569463548830814</v>
+        <v>4.8486932599724906</v>
       </c>
     </row>
     <row r="33" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C33" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D33" t="s">
         <v>81</v>
       </c>
       <c r="E33" s="11">
-        <v>2.9881895365934641</v>
+        <v>2.9917469050894088</v>
       </c>
     </row>
     <row r="34" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C34" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D34" t="s">
         <v>81</v>
       </c>
       <c r="E34" s="11">
-        <v>0.64032632927002808</v>
+        <v>6.5064269790826748</v>
       </c>
     </row>
     <row r="35" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C35" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="D35" t="s">
         <v>81</v>
       </c>
       <c r="E35" s="11">
-        <v>2.7854195323246222</v>
+        <v>18.569463548830814</v>
       </c>
     </row>
     <row r="36" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C36" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D36" t="s">
         <v>81</v>
       </c>
       <c r="E36" s="11">
+        <v>2.9881895365934641</v>
+      </c>
+    </row>
+    <row r="37" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C37" t="s">
+        <v>89</v>
+      </c>
+      <c r="D37" t="s">
+        <v>81</v>
+      </c>
+      <c r="E37" s="11">
+        <v>0.64032632927002808</v>
+      </c>
+    </row>
+    <row r="38" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C38" t="s">
+        <v>98</v>
+      </c>
+      <c r="D38" t="s">
+        <v>81</v>
+      </c>
+      <c r="E38" s="11">
+        <v>2.7854195323246222</v>
+      </c>
+    </row>
+    <row r="39" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C39" t="s">
+        <v>90</v>
+      </c>
+      <c r="D39" t="s">
+        <v>81</v>
+      </c>
+      <c r="E39" s="11">
         <v>1.66010529810748</v>
       </c>
-      <c r="G36" s="15" t="s">
+      <c r="G39" s="15" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="37" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C37" s="15" t="s">
+    <row r="40" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C40" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="E37" s="11"/>
-    </row>
-    <row r="38" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C38" s="15" t="s">
+      <c r="E40" s="11"/>
+    </row>
+    <row r="41" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C41" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="E38" s="11"/>
+      <c r="E41" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>